<commit_message>
Anchor charts in genuinely empty space; guard against chart-over-content overlap
Header bands were painted 11-13 columns wide while their tables used
3-4, and each block's chart was anchored inside the painted band.
Bands are now as wide as their tables, per-indicator chart y-axes get
a compact tick format, and a new check walks every chart's anchor
extent (EMU size over real column/row dimensions) and fails if it
covers any cell with a value or fill: Indicator Check 484->0,
New Data Overview 6->0, Combined 490->0. 44 checks pass.

Claude-Session: https://claude.ai/code/session_01CMyfpFes85KZq9gRWwC3V4
</commit_message>
<xml_diff>
--- a/project-documents/summer-prep-background/ESABCC_Indicator-New-Data-Overview_2026-07.xlsx
+++ b/project-documents/summer-prep-background/ESABCC_Indicator-New-Data-Overview_2026-07.xlsx
@@ -4354,13 +4354,6 @@
           <t>Still at the report figure</t>
         </is>
       </c>
-      <c r="E66" s="4" t="inlineStr"/>
-      <c r="F66" s="4" t="inlineStr"/>
-      <c r="G66" s="4" t="inlineStr"/>
-      <c r="H66" s="4" t="inlineStr"/>
-      <c r="I66" s="4" t="inlineStr"/>
-      <c r="J66" s="4" t="inlineStr"/>
-      <c r="K66" s="4" t="inlineStr"/>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" s="6" t="inlineStr"/>

</xml_diff>